<commit_message>
siddyq 7-5 finshing befor ly mod
</commit_message>
<xml_diff>
--- a/puruch list/Copy of perch_list(1).xlsx
+++ b/puruch list/Copy of perch_list(1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morga\OneDrive\project\robocheel\mineSweper\puruch list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA724CA8-733C-4CBE-A601-C6BCF110D0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D1C3A6-3169-4585-9E66-6ADE5F923B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BA8BC2EA-4C6A-4475-BE7E-C15009A97951}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{BA8BC2EA-4C6A-4475-BE7E-C15009A97951}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
   <si>
     <t>esp32</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -685,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05AE4299-62B9-4A3F-BF02-744309EC2A9B}">
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.1796875" customWidth="1"/>
@@ -693,7 +696,7 @@
     <col min="4" max="4" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -710,8 +713,11 @@
         <f>D1*B1</f>
         <v>600</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -729,7 +735,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -747,7 +753,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -765,7 +771,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -783,7 +789,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -801,7 +807,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -819,7 +825,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -837,7 +843,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -855,7 +861,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -873,7 +879,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -891,7 +897,7 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -909,7 +915,7 @@
         <v>62.5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -927,7 +933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -945,7 +951,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -963,7 +969,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>

</xml_diff>